<commit_message>
Incorpora la valoración de las coordinaciones a la evaluación (paso 8)
</commit_message>
<xml_diff>
--- a/docs/evaluacion/material-coordinaciones/GH-seg-2425/rubrica-valoracion.xlsx
+++ b/docs/evaluacion/material-coordinaciones/GH-seg-2425/rubrica-valoracion.xlsx
@@ -65,7 +65,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -87,11 +87,55 @@
         <color rgb="00C5CED9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C5CED9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C5CED9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C5CED9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C5CED9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C5CED9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C5CED9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C5CED9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C5CED9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -123,6 +167,8 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -488,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -511,14 +557,14 @@
           <t>Título</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
+      <c r="B3" s="15" t="n"/>
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Grado en Historia</t>
         </is>
       </c>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
+      <c r="D3" s="16" t="n"/>
+      <c r="E3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -526,14 +572,14 @@
           <t>Autoinforme</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
+      <c r="B4" s="15" t="n"/>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Seguimiento, curso 2024/25 (convocatoria 2026)</t>
         </is>
       </c>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
+      <c r="D4" s="16" t="n"/>
+      <c r="E4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -541,10 +587,10 @@
           <t>Rol de quien valora</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n"/>
+      <c r="B5" s="15" t="n"/>
       <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="15" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -552,15 +598,15 @@
           <t>Fecha</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n"/>
+      <c r="B6" s="15" t="n"/>
       <c r="C6" s="4" t="inlineStr"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="15" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Escala: 1 = hay que rehacerlo · 3 = aprovechable corrigiendo o completando partes relevantes · 5 = utilizable casi sin cambios.</t>
+          <t>Escala: 1 = hay que rehacerlo · 3 = aprovechable corrigiendo o completando partes relevantes · 5 = utilizable casi sin cambios. Deje en blanco los aspectos que no apliquen.</t>
         </is>
       </c>
     </row>
@@ -597,12 +643,12 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Datos</t>
+          <t>Identificación</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>¿Son correctos los datos del título y los indicadores?</t>
+          <t>¿Son correctos los datos de identificación del título (denominación, centro, créditos, plazas, modalidad…)?</t>
         </is>
       </c>
       <c r="D11" s="8" t="n"/>
@@ -614,12 +660,12 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Cobertura</t>
+          <t>Indicadores</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>¿Trata todos los apartados que exige la plantilla?</t>
+          <t>¿Son correctos los valores de los indicadores y están bien alineados con sus cursos y cohortes?</t>
         </is>
       </c>
       <c r="D12" s="8" t="n"/>
@@ -631,12 +677,12 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Análisis</t>
+          <t>Cobertura</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>¿La interpretación de los resultados es acertada y útil para el título?</t>
+          <t>¿Trata todos los apartados que exige la plantilla?</t>
         </is>
       </c>
       <c r="D13" s="8" t="n"/>
@@ -648,12 +694,12 @@
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Mejora</t>
+          <t>Análisis</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>¿Los puntos fuertes, los puntos débiles y el plan de mejora son realistas y asumibles?</t>
+          <t>¿La interpretación de los resultados es acertada y útil para el título?</t>
         </is>
       </c>
       <c r="D14" s="8" t="n"/>
@@ -665,29 +711,29 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Redacción</t>
+          <t>Mejora</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>¿El estilo y el formato son adecuados para entregarlo tras revisarlo?</t>
+          <t>¿Los puntos fuertes, los puntos débiles y el plan de mejora son realistas y asumibles?</t>
         </is>
       </c>
       <c r="D15" s="8" t="n"/>
       <c r="E15" s="9" t="n"/>
     </row>
-    <row r="16" ht="32" customHeight="1">
+    <row r="16" ht="48" customHeight="1">
       <c r="A16" s="10" t="n">
         <v>6</v>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Esfuerzo</t>
+          <t>Recomendaciones</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>¿Revisarlo y completarlo cuesta menos que elaborarlo desde cero?</t>
+          <t>¿Recoge todas las recomendaciones vigentes de la agencia (ACCUA/DEVA), con su numeración original y su estado o acción? Déjelo en blanco si el título no tiene recomendaciones.</t>
         </is>
       </c>
       <c r="D16" s="8" t="n"/>
@@ -699,72 +745,125 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Global</t>
+          <t>Redacción</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>¿Lo usaría como punto de partida para el próximo autoinforme?</t>
+          <t>¿El estilo y el formato son adecuados para entregarlo tras revisarlo?</t>
         </is>
       </c>
       <c r="D17" s="8" t="n"/>
       <c r="E17" s="9" t="n"/>
     </row>
-    <row r="18">
-      <c r="C18" s="11" t="inlineStr">
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Esfuerzo</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>¿Revisarlo y completarlo cuesta menos que elaborarlo desde cero?</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="9" t="n"/>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>¿Lo usaría como punto de partida para el próximo autoinforme?</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="9" t="n"/>
+    </row>
+    <row r="20">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="D18" s="12">
-        <f>IFERROR(ROUND(AVERAGE(D11:D17),2),"")</f>
+      <c r="D20" s="12">
+        <f>IFERROR(ROUND(AVERAGE(D11:D19),2),"")</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+    <row r="22" ht="64" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>!</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Errores graves</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>¿Ha encontrado algún dato inventado (sin origen en la documentación ni en los indicadores oficiales) o contradictorio (un valor imposible o el mismo indicador con dos valores distintos)? Indique cuáles en el comentario.</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="9" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>¿Qué cambiaría del borrador?</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="9" t="n"/>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="9" t="n"/>
+      <c r="B25" s="16" t="n"/>
+      <c r="C25" s="16" t="n"/>
+      <c r="D25" s="16" t="n"/>
+      <c r="E25" s="15" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>¿Qué echa en falta?</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1">
-      <c r="A24" s="9" t="n"/>
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+    <row r="28" ht="60" customHeight="1">
+      <c r="A28" s="9" t="n"/>
+      <c r="B28" s="16" t="n"/>
+      <c r="C28" s="16" t="n"/>
+      <c r="D28" s="16" t="n"/>
+      <c r="E28" s="15" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
         <is>
           <t>Otros comentarios</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1">
-      <c r="A27" s="9" t="n"/>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="14" t="inlineStr">
+    <row r="31" ht="60" customHeight="1">
+      <c r="A31" s="9" t="n"/>
+      <c r="B31" s="16" t="n"/>
+      <c r="C31" s="16" t="n"/>
+      <c r="D31" s="16" t="n"/>
+      <c r="E31" s="15" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t>Rellene las celdas en amarillo.</t>
         </is>
@@ -772,27 +871,30 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A21:E21"/>
-    <mergeCell ref="A20:E20"/>
-    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="A30:E30"/>
     <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A26:E26"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C4:E4"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C3:E3"/>
-    <mergeCell ref="A23:E23"/>
     <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:E6"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="A31:E31"/>
     <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A6:B6"/>
     <mergeCell ref="A27:E27"/>
-    <mergeCell ref="C6:E6"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="D11 D12 D13 D14 D15 D16 D17" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Introduce un número entero del 1 al 5." type="whole" operator="between">
+  <dataValidations count="2">
+    <dataValidation sqref="D11:D19" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Introduce un número entero del 1 al 5." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation sqref="D22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Elige Sí o No." type="list">
+      <formula1>"Sí,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>